<commit_message>
docs: fill in test placeholder phone numbers for the carrier customers
Real numbers still needed before this is a permanent record — flagged in the
Notes column.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/MERCON_Customers_ReadyToImport_Carriers.xlsx
+++ b/docs/templates/MERCON_Customers_ReadyToImport_Carriers.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
   <si>
     <t>MERCON LOGISTICS — CARRIER CUSTOMERS (from COMPANY QUOTATION.xlsx)</t>
   </si>
@@ -31,28 +31,46 @@
     <t>JDL</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Fill in phone before importing</t>
+    <t>966500000001</t>
+  </si>
+  <si>
+    <t>TEST placeholder phone — replace with the real number</t>
   </si>
   <si>
     <t>IMILE</t>
   </si>
   <si>
+    <t>966500000002</t>
+  </si>
+  <si>
     <t>SHIPA</t>
   </si>
   <si>
+    <t>966500000003</t>
+  </si>
+  <si>
     <t>RTL</t>
   </si>
   <si>
+    <t>966500000004</t>
+  </si>
+  <si>
     <t>HORIZON</t>
   </si>
   <si>
+    <t>966500000005</t>
+  </si>
+  <si>
     <t>ARKAN BARWAN</t>
   </si>
   <si>
+    <t>966500000006</t>
+  </si>
+  <si>
     <t>AKS</t>
+  </si>
+  <si>
+    <t>966500000007</t>
   </si>
 </sst>
 </file>
@@ -514,7 +532,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C6" t="s">
         <v>7</v>
@@ -522,10 +540,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
         <v>7</v>
@@ -533,10 +551,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
         <v>7</v>
@@ -544,10 +562,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
         <v>7</v>
@@ -555,10 +573,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="C10" t="s">
         <v>7</v>
@@ -566,10 +584,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C11" t="s">
         <v>7</v>
@@ -581,6 +599,6 @@
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>